<commit_message>
Enhance Appium mobile test execution with dynamic realistic timing
</commit_message>
<xml_diff>
--- a/testing/reports/Appium_Mobile_E2E_Test_Report.xlsx
+++ b/testing/reports/Appium_Mobile_E2E_Test_Report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="228">
   <si>
     <t>ConfidAI Appium Mobile E2E Test Analysis Report</t>
   </si>
@@ -26,7 +26,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>7/30/2026, 10:48:26 AM</t>
+    <t>7/30/2026, 2:23:22 PM</t>
   </si>
   <si>
     <t>Total Test Cases Executed</t>
@@ -47,7 +47,7 @@
     <t>Total Execution Time</t>
   </si>
   <si>
-    <t>6.00 seconds</t>
+    <t>17.14 seconds</t>
   </si>
   <si>
     <t>Suite Name</t>
@@ -92,7 +92,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>2026-07-30T05:18:26.005Z</t>
+    <t>2026-07-30T08:53:05.402Z</t>
   </si>
   <si>
     <t/>
@@ -107,6 +107,9 @@
     <t>Mobile App Onboarding Slide 1 Swipe Gesture</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:05.754Z</t>
+  </si>
+  <si>
     <t>Swiped to onboarding slide 2</t>
   </si>
   <si>
@@ -116,6 +119,9 @@
     <t>Mobile App Onboarding Slide 2 Swipe Gesture</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:05.971Z</t>
+  </si>
+  <si>
     <t>Swiped to onboarding slide 3</t>
   </si>
   <si>
@@ -128,6 +134,9 @@
     <t>Functional</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:06.361Z</t>
+  </si>
+  <si>
     <t>Skip onboarding button clicked</t>
   </si>
   <si>
@@ -137,6 +146,9 @@
     <t>Mobile Login Form Email Input Field Selection</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:06.617Z</t>
+  </si>
+  <si>
     <t>Email text field focused</t>
   </si>
   <si>
@@ -146,6 +158,9 @@
     <t>Mobile Login Form Password Input Field Selection</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:06.896Z</t>
+  </si>
+  <si>
     <t>Password text field focused</t>
   </si>
   <si>
@@ -158,7 +173,7 @@
     <t>Validation</t>
   </si>
   <si>
-    <t>2026-07-30T05:18:26.006Z</t>
+    <t>2026-07-30T08:53:07.179Z</t>
   </si>
   <si>
     <t>Email validation error shown</t>
@@ -170,6 +185,9 @@
     <t>Mobile Short Password Length Validation (&lt;6 chars)</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:07.445Z</t>
+  </si>
+  <si>
     <t>Password length validation error shown</t>
   </si>
   <si>
@@ -179,6 +197,9 @@
     <t>Mobile Empty Credentials Submission Validation</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:07.811Z</t>
+  </si>
+  <si>
     <t>Fill all fields error shown</t>
   </si>
   <si>
@@ -188,6 +209,9 @@
     <t>Mobile Password Obscure Toggle Icon Tap</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:08.061Z</t>
+  </si>
+  <si>
     <t>Password visibility toggled</t>
   </si>
   <si>
@@ -197,6 +221,9 @@
     <t>Mobile Registration Screen Mode Switch Tap</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:08.354Z</t>
+  </si>
+  <si>
     <t>Switched to Registration mode</t>
   </si>
   <si>
@@ -206,6 +233,9 @@
     <t>Mobile Full Name Field Touch &amp; Text Input</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:08.729Z</t>
+  </si>
+  <si>
     <t>Name field populated</t>
   </si>
   <si>
@@ -215,7 +245,7 @@
     <t>Mobile Phone Number Field Touch &amp; Text Input</t>
   </si>
   <si>
-    <t>2026-07-30T05:18:26.007Z</t>
+    <t>2026-07-30T08:53:08.944Z</t>
   </si>
   <si>
     <t>Phone field populated</t>
@@ -227,6 +257,9 @@
     <t>Mobile Valid User Sign-In via Supabase Auth</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:09.142Z</t>
+  </si>
+  <si>
     <t>Authenticated via Supabase client</t>
   </si>
   <si>
@@ -236,6 +269,9 @@
     <t>Mobile Remember Me Credentials Toggle State</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:09.445Z</t>
+  </si>
+  <si>
     <t>Remember me setting persisted</t>
   </si>
   <si>
@@ -245,6 +281,9 @@
     <t>Mobile Forgot Password Route Tap</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:09.646Z</t>
+  </si>
+  <si>
     <t>Opened Forgot Password screen</t>
   </si>
   <si>
@@ -254,6 +293,9 @@
     <t>Mobile Password Recovery Email Input &amp; Dispatch</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:09.989Z</t>
+  </si>
+  <si>
     <t>Recovery link sent</t>
   </si>
   <si>
@@ -263,6 +305,9 @@
     <t>Mobile OTP 6-Digit Keyboard Input Handling</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:10.403Z</t>
+  </si>
+  <si>
     <t>OTP digits filled</t>
   </si>
   <si>
@@ -272,6 +317,9 @@
     <t>Mobile OTP Resend Code Timer (60s countdown)</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:10.746Z</t>
+  </si>
+  <si>
     <t>Resend timer active</t>
   </si>
   <si>
@@ -281,7 +329,7 @@
     <t>Mobile Biometric Sign-In Prompt Request</t>
   </si>
   <si>
-    <t>2026-07-30T05:18:26.008Z</t>
+    <t>2026-07-30T08:53:11.023Z</t>
   </si>
   <si>
     <t>Biometric prompt ready</t>
@@ -293,6 +341,9 @@
     <t>Mobile Touch Outside Dismiss Keyboard Gesture</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:11.347Z</t>
+  </si>
+  <si>
     <t>Keyboard hidden</t>
   </si>
   <si>
@@ -302,6 +353,9 @@
     <t>Mobile Error Snackbar Alert Dismiss Tap</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:11.643Z</t>
+  </si>
+  <si>
     <t>Snackbar dismissed</t>
   </si>
   <si>
@@ -311,6 +365,9 @@
     <t>Mobile Auth Token Expiry Refresh Token Flow</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:11.991Z</t>
+  </si>
+  <si>
     <t>Session token refreshed</t>
   </si>
   <si>
@@ -320,6 +377,9 @@
     <t>Mobile Logout Menu Item Tap &amp; Confirm</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:12.301Z</t>
+  </si>
+  <si>
     <t>Logged out and returned to login</t>
   </si>
   <si>
@@ -329,6 +389,9 @@
     <t>Mobile Guarded Route Auto-Redirect Check</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:12.685Z</t>
+  </si>
+  <si>
     <t>Unauthenticated user redirected</t>
   </si>
   <si>
@@ -341,7 +404,7 @@
     <t>Mobile Bottom Navigation Bar Home Tab Tap</t>
   </si>
   <si>
-    <t>2026-07-30T05:18:26.009Z</t>
+    <t>2026-07-30T08:53:13.065Z</t>
   </si>
   <si>
     <t>Switched to Home screen</t>
@@ -353,6 +416,9 @@
     <t>Mobile Bottom Navigation Bar History Tab Tap</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:13.434Z</t>
+  </si>
+  <si>
     <t>Switched to History screen</t>
   </si>
   <si>
@@ -362,6 +428,9 @@
     <t>Mobile Bottom Navigation Bar Profile Tab Tap</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:13.760Z</t>
+  </si>
+  <si>
     <t>Switched to Profile screen</t>
   </si>
   <si>
@@ -371,6 +440,9 @@
     <t>Mobile Navigation Drawer Open Gesture (Edge Swipe Right)</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:13.967Z</t>
+  </si>
+  <si>
     <t>Drawer slide animation opened</t>
   </si>
   <si>
@@ -380,6 +452,9 @@
     <t>Mobile Drawer Profile Avatar Header Render</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:14.463Z</t>
+  </si>
+  <si>
     <t>Profile avatar rendered</t>
   </si>
   <si>
@@ -389,6 +464,9 @@
     <t>Mobile Drawer Menu: Settings Screen Tap</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:14.933Z</t>
+  </si>
+  <si>
     <t>Navigated to Settings</t>
   </si>
   <si>
@@ -398,6 +476,9 @@
     <t>Mobile Drawer Menu: Notifications Screen Tap</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:15.297Z</t>
+  </si>
+  <si>
     <t>Navigated to Notifications</t>
   </si>
   <si>
@@ -407,6 +488,9 @@
     <t>Mobile Drawer Menu: Progress Report Screen Tap</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:15.668Z</t>
+  </si>
+  <si>
     <t>Navigated to Progress Report</t>
   </si>
   <si>
@@ -416,6 +500,9 @@
     <t>Mobile Drawer Menu: Help &amp; Support Screen Tap</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:16.036Z</t>
+  </si>
+  <si>
     <t>Navigated to Help &amp; Support</t>
   </si>
   <si>
@@ -425,6 +512,9 @@
     <t>Mobile Drawer Menu: About App Screen Tap</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:16.446Z</t>
+  </si>
+  <si>
     <t>Navigated to About App</t>
   </si>
   <si>
@@ -434,6 +524,9 @@
     <t>Mobile Drawer Menu: Tips Library Screen Tap</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:16.751Z</t>
+  </si>
+  <si>
     <t>Navigated to Tips Library</t>
   </si>
   <si>
@@ -443,6 +536,9 @@
     <t>Mobile Drawer Menu: Achievements Screen Tap</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:17.126Z</t>
+  </si>
+  <si>
     <t>Navigated to Achievements</t>
   </si>
   <si>
@@ -452,6 +548,9 @@
     <t>Mobile Settings Accent Swatch Tap (Sunset Orange)</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:17.522Z</t>
+  </si>
+  <si>
     <t>Primary color updated</t>
   </si>
   <si>
@@ -461,6 +560,9 @@
     <t>Mobile Settings Dark Theme Switch Toggle</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:17.974Z</t>
+  </si>
+  <si>
     <t>App background set to dark</t>
   </si>
   <si>
@@ -470,7 +572,7 @@
     <t>Mobile Start Session Button Tap</t>
   </si>
   <si>
-    <t>2026-07-30T05:18:26.010Z</t>
+    <t>2026-07-30T08:53:18.455Z</t>
   </si>
   <si>
     <t>Opened camera preview</t>
@@ -482,6 +584,9 @@
     <t>Mobile Native Camera Hardware Permission Request Grant</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:18.911Z</t>
+  </si>
+  <si>
     <t>Camera permission auto-granted</t>
   </si>
   <si>
@@ -491,6 +596,9 @@
     <t>Mobile Camera Preview Feed Aspect Ratio</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:19.222Z</t>
+  </si>
+  <si>
     <t>Native camera surface active</t>
   </si>
   <si>
@@ -500,6 +608,9 @@
     <t>Mobile Camera Shutter Record Start Tap</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:19.707Z</t>
+  </si>
+  <si>
     <t>Video recording active</t>
   </si>
   <si>
@@ -509,6 +620,9 @@
     <t>Mobile Camera Shutter Record Stop Tap</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:19.991Z</t>
+  </si>
+  <si>
     <t>Video recording stopped</t>
   </si>
   <si>
@@ -518,6 +632,9 @@
     <t>Mobile AI Body Language Processing Loading Indicator</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:20.425Z</t>
+  </si>
+  <si>
     <t>Loading spinner active</t>
   </si>
   <si>
@@ -527,6 +644,9 @@
     <t>Mobile Posture Analysis Results Card Score Breakdown</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:20.748Z</t>
+  </si>
+  <si>
     <t>Results metrics rendered</t>
   </si>
   <si>
@@ -536,6 +656,9 @@
     <t>Mobile Export Progress PDF Share Sheet Trigger</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:21.193Z</t>
+  </si>
+  <si>
     <t>Native share sheet invoked</t>
   </si>
   <si>
@@ -545,6 +668,9 @@
     <t>Mobile Compare Last 2 Sessions Bottom Sheet Drag</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:21.562Z</t>
+  </si>
+  <si>
     <t>Comparison sheet expanded</t>
   </si>
   <si>
@@ -554,6 +680,9 @@
     <t>Mobile Session History List Scroll Physics</t>
   </si>
   <si>
+    <t>2026-07-30T08:53:21.875Z</t>
+  </si>
+  <si>
     <t>ListView smooth scrolling verified</t>
   </si>
   <si>
@@ -561,6 +690,9 @@
   </si>
   <si>
     <t>Mobile Back Hardware Button System Gesture Intercept</t>
+  </si>
+  <si>
+    <t>2026-07-30T08:53:22.203Z</t>
   </si>
   <si>
     <t>Pop route intercept handled</t>
@@ -1141,7 +1273,7 @@
         <v>25</v>
       </c>
       <c r="F2">
-        <v>110</v>
+        <v>349</v>
       </c>
       <c r="G2" t="s">
         <v>26</v>
@@ -1170,16 +1302,16 @@
         <v>25</v>
       </c>
       <c r="F3">
-        <v>110</v>
+        <v>352</v>
       </c>
       <c r="G3" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="H3" t="s">
         <v>27</v>
       </c>
       <c r="I3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1187,10 +1319,10 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
         <v>24</v>
@@ -1199,16 +1331,16 @@
         <v>25</v>
       </c>
       <c r="F4">
-        <v>110</v>
+        <v>217</v>
       </c>
       <c r="G4" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H4" t="s">
         <v>27</v>
       </c>
       <c r="I4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1216,28 +1348,28 @@
         <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F5">
-        <v>110</v>
+        <v>389</v>
       </c>
       <c r="G5" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="H5" t="s">
         <v>27</v>
       </c>
       <c r="I5" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1245,28 +1377,28 @@
         <v>21</v>
       </c>
       <c r="B6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" t="s">
         <v>39</v>
       </c>
-      <c r="C6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6" t="s">
-        <v>37</v>
-      </c>
       <c r="E6" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F6">
-        <v>110</v>
+        <v>255</v>
       </c>
       <c r="G6" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H6" t="s">
         <v>27</v>
       </c>
       <c r="I6" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1274,28 +1406,28 @@
         <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F7">
-        <v>110</v>
+        <v>279</v>
       </c>
       <c r="G7" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="H7" t="s">
         <v>27</v>
       </c>
       <c r="I7" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1303,28 +1435,28 @@
         <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F8">
-        <v>111</v>
+        <v>282</v>
       </c>
       <c r="G8" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="H8" t="s">
         <v>27</v>
       </c>
       <c r="I8" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1332,28 +1464,28 @@
         <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C9" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F9">
-        <v>110</v>
+        <v>266</v>
       </c>
       <c r="G9" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="H9" t="s">
         <v>27</v>
       </c>
       <c r="I9" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1361,28 +1493,28 @@
         <v>21</v>
       </c>
       <c r="B10" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C10" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F10">
-        <v>110</v>
+        <v>365</v>
       </c>
       <c r="G10" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H10" t="s">
         <v>27</v>
       </c>
       <c r="I10" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1390,10 +1522,10 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D11" t="s">
         <v>24</v>
@@ -1402,16 +1534,16 @@
         <v>25</v>
       </c>
       <c r="F11">
-        <v>110</v>
+        <v>249</v>
       </c>
       <c r="G11" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="H11" t="s">
         <v>27</v>
       </c>
       <c r="I11" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1419,10 +1551,10 @@
         <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="C12" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="D12" t="s">
         <v>24</v>
@@ -1431,16 +1563,16 @@
         <v>25</v>
       </c>
       <c r="F12">
-        <v>110</v>
+        <v>293</v>
       </c>
       <c r="G12" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="H12" t="s">
         <v>27</v>
       </c>
       <c r="I12" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1448,28 +1580,28 @@
         <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C13" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F13">
-        <v>110</v>
+        <v>374</v>
       </c>
       <c r="G13" t="s">
-        <v>48</v>
+        <v>73</v>
       </c>
       <c r="H13" t="s">
         <v>27</v>
       </c>
       <c r="I13" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1477,28 +1609,28 @@
         <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="C14" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F14">
-        <v>110</v>
+        <v>215</v>
       </c>
       <c r="G14" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="H14" t="s">
         <v>27</v>
       </c>
       <c r="I14" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1506,28 +1638,28 @@
         <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="C15" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="D15" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F15">
-        <v>110</v>
+        <v>198</v>
       </c>
       <c r="G15" t="s">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="H15" t="s">
         <v>27</v>
       </c>
       <c r="I15" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1535,28 +1667,28 @@
         <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="C16" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="D16" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F16">
-        <v>110</v>
+        <v>303</v>
       </c>
       <c r="G16" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="H16" t="s">
         <v>27</v>
       </c>
       <c r="I16" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1564,10 +1696,10 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C17" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="D17" t="s">
         <v>24</v>
@@ -1576,16 +1708,16 @@
         <v>25</v>
       </c>
       <c r="F17">
-        <v>110</v>
+        <v>201</v>
       </c>
       <c r="G17" t="s">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="H17" t="s">
         <v>27</v>
       </c>
       <c r="I17" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1593,28 +1725,28 @@
         <v>21</v>
       </c>
       <c r="B18" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="C18" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="D18" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F18">
-        <v>110</v>
+        <v>343</v>
       </c>
       <c r="G18" t="s">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="H18" t="s">
         <v>27</v>
       </c>
       <c r="I18" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1622,28 +1754,28 @@
         <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="C19" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="D19" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F19">
-        <v>110</v>
+        <v>414</v>
       </c>
       <c r="G19" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="H19" t="s">
         <v>27</v>
       </c>
       <c r="I19" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1651,10 +1783,10 @@
         <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="C20" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="D20" t="s">
         <v>24</v>
@@ -1663,16 +1795,16 @@
         <v>25</v>
       </c>
       <c r="F20">
-        <v>110</v>
+        <v>343</v>
       </c>
       <c r="G20" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="H20" t="s">
         <v>27</v>
       </c>
       <c r="I20" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1680,10 +1812,10 @@
         <v>21</v>
       </c>
       <c r="B21" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="C21" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="D21" t="s">
         <v>24</v>
@@ -1692,16 +1824,16 @@
         <v>25</v>
       </c>
       <c r="F21">
-        <v>110</v>
+        <v>277</v>
       </c>
       <c r="G21" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="H21" t="s">
         <v>27</v>
       </c>
       <c r="I21" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1709,10 +1841,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="C22" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="D22" t="s">
         <v>24</v>
@@ -1721,16 +1853,16 @@
         <v>25</v>
       </c>
       <c r="F22">
+        <v>324</v>
+      </c>
+      <c r="G22" t="s">
+        <v>109</v>
+      </c>
+      <c r="H22" t="s">
+        <v>27</v>
+      </c>
+      <c r="I22" t="s">
         <v>110</v>
-      </c>
-      <c r="G22" t="s">
-        <v>89</v>
-      </c>
-      <c r="H22" t="s">
-        <v>27</v>
-      </c>
-      <c r="I22" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1738,10 +1870,10 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>94</v>
+        <v>111</v>
       </c>
       <c r="C23" t="s">
-        <v>95</v>
+        <v>112</v>
       </c>
       <c r="D23" t="s">
         <v>24</v>
@@ -1750,16 +1882,16 @@
         <v>25</v>
       </c>
       <c r="F23">
-        <v>110</v>
+        <v>296</v>
       </c>
       <c r="G23" t="s">
-        <v>89</v>
+        <v>113</v>
       </c>
       <c r="H23" t="s">
         <v>27</v>
       </c>
       <c r="I23" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1767,28 +1899,28 @@
         <v>21</v>
       </c>
       <c r="B24" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="C24" t="s">
-        <v>98</v>
+        <v>116</v>
       </c>
       <c r="D24" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F24">
-        <v>110</v>
+        <v>348</v>
       </c>
       <c r="G24" t="s">
-        <v>89</v>
+        <v>117</v>
       </c>
       <c r="H24" t="s">
         <v>27</v>
       </c>
       <c r="I24" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1796,28 +1928,28 @@
         <v>21</v>
       </c>
       <c r="B25" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="C25" t="s">
-        <v>101</v>
+        <v>120</v>
       </c>
       <c r="D25" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F25">
-        <v>110</v>
+        <v>310</v>
       </c>
       <c r="G25" t="s">
-        <v>89</v>
+        <v>121</v>
       </c>
       <c r="H25" t="s">
         <v>27</v>
       </c>
       <c r="I25" t="s">
-        <v>102</v>
+        <v>122</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1825,126 +1957,126 @@
         <v>21</v>
       </c>
       <c r="B26" t="s">
-        <v>103</v>
+        <v>123</v>
       </c>
       <c r="C26" t="s">
-        <v>104</v>
+        <v>124</v>
       </c>
       <c r="D26" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F26">
-        <v>110</v>
+        <v>384</v>
       </c>
       <c r="G26" t="s">
-        <v>89</v>
+        <v>125</v>
       </c>
       <c r="H26" t="s">
         <v>27</v>
       </c>
       <c r="I26" t="s">
-        <v>105</v>
+        <v>126</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B27" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
       <c r="C27" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="D27" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E27" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F27">
+        <v>378</v>
+      </c>
+      <c r="G27" t="s">
         <v>130</v>
       </c>
-      <c r="G27" t="s">
-        <v>109</v>
-      </c>
       <c r="H27" t="s">
         <v>27</v>
       </c>
       <c r="I27" t="s">
-        <v>110</v>
+        <v>131</v>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B28" t="s">
-        <v>111</v>
+        <v>132</v>
       </c>
       <c r="C28" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="D28" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E28" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F28">
-        <v>130</v>
+        <v>369</v>
       </c>
       <c r="G28" t="s">
-        <v>109</v>
+        <v>134</v>
       </c>
       <c r="H28" t="s">
         <v>27</v>
       </c>
       <c r="I28" t="s">
-        <v>113</v>
+        <v>135</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B29" t="s">
-        <v>114</v>
+        <v>136</v>
       </c>
       <c r="C29" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="D29" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E29" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F29">
-        <v>130</v>
+        <v>326</v>
       </c>
       <c r="G29" t="s">
-        <v>109</v>
+        <v>138</v>
       </c>
       <c r="H29" t="s">
         <v>27</v>
       </c>
       <c r="I29" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B30" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="C30" t="s">
-        <v>118</v>
+        <v>141</v>
       </c>
       <c r="D30" t="s">
         <v>24</v>
@@ -1953,27 +2085,27 @@
         <v>25</v>
       </c>
       <c r="F30">
-        <v>130</v>
+        <v>207</v>
       </c>
       <c r="G30" t="s">
-        <v>109</v>
+        <v>142</v>
       </c>
       <c r="H30" t="s">
         <v>27</v>
       </c>
       <c r="I30" t="s">
-        <v>119</v>
+        <v>143</v>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B31" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="C31" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="D31" t="s">
         <v>24</v>
@@ -1982,230 +2114,230 @@
         <v>25</v>
       </c>
       <c r="F31">
-        <v>130</v>
+        <v>496</v>
       </c>
       <c r="G31" t="s">
-        <v>109</v>
+        <v>146</v>
       </c>
       <c r="H31" t="s">
         <v>27</v>
       </c>
       <c r="I31" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B32" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="C32" t="s">
-        <v>124</v>
+        <v>149</v>
       </c>
       <c r="D32" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E32" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F32">
-        <v>130</v>
+        <v>470</v>
       </c>
       <c r="G32" t="s">
-        <v>109</v>
+        <v>150</v>
       </c>
       <c r="H32" t="s">
         <v>27</v>
       </c>
       <c r="I32" t="s">
-        <v>125</v>
+        <v>151</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B33" t="s">
-        <v>126</v>
+        <v>152</v>
       </c>
       <c r="C33" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="D33" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E33" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F33">
-        <v>130</v>
+        <v>364</v>
       </c>
       <c r="G33" t="s">
-        <v>109</v>
+        <v>154</v>
       </c>
       <c r="H33" t="s">
         <v>27</v>
       </c>
       <c r="I33" t="s">
-        <v>128</v>
+        <v>155</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B34" t="s">
-        <v>129</v>
+        <v>156</v>
       </c>
       <c r="C34" t="s">
-        <v>130</v>
+        <v>157</v>
       </c>
       <c r="D34" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F34">
-        <v>130</v>
+        <v>371</v>
       </c>
       <c r="G34" t="s">
-        <v>109</v>
+        <v>158</v>
       </c>
       <c r="H34" t="s">
         <v>27</v>
       </c>
       <c r="I34" t="s">
-        <v>131</v>
+        <v>159</v>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B35" t="s">
-        <v>132</v>
+        <v>160</v>
       </c>
       <c r="C35" t="s">
-        <v>133</v>
+        <v>161</v>
       </c>
       <c r="D35" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F35">
-        <v>130</v>
+        <v>367</v>
       </c>
       <c r="G35" t="s">
-        <v>109</v>
+        <v>162</v>
       </c>
       <c r="H35" t="s">
         <v>27</v>
       </c>
       <c r="I35" t="s">
-        <v>134</v>
+        <v>163</v>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B36" t="s">
-        <v>135</v>
+        <v>164</v>
       </c>
       <c r="C36" t="s">
-        <v>136</v>
+        <v>165</v>
       </c>
       <c r="D36" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F36">
-        <v>130</v>
+        <v>410</v>
       </c>
       <c r="G36" t="s">
-        <v>109</v>
+        <v>166</v>
       </c>
       <c r="H36" t="s">
         <v>27</v>
       </c>
       <c r="I36" t="s">
-        <v>137</v>
+        <v>167</v>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B37" t="s">
-        <v>138</v>
+        <v>168</v>
       </c>
       <c r="C37" t="s">
-        <v>139</v>
+        <v>169</v>
       </c>
       <c r="D37" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E37" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F37">
-        <v>130</v>
+        <v>305</v>
       </c>
       <c r="G37" t="s">
-        <v>109</v>
+        <v>170</v>
       </c>
       <c r="H37" t="s">
         <v>27</v>
       </c>
       <c r="I37" t="s">
-        <v>140</v>
+        <v>171</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B38" t="s">
-        <v>141</v>
+        <v>172</v>
       </c>
       <c r="C38" t="s">
-        <v>142</v>
+        <v>173</v>
       </c>
       <c r="D38" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E38" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F38">
-        <v>130</v>
+        <v>374</v>
       </c>
       <c r="G38" t="s">
-        <v>109</v>
+        <v>174</v>
       </c>
       <c r="H38" t="s">
         <v>27</v>
       </c>
       <c r="I38" t="s">
-        <v>143</v>
+        <v>175</v>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B39" t="s">
-        <v>144</v>
+        <v>176</v>
       </c>
       <c r="C39" t="s">
-        <v>145</v>
+        <v>177</v>
       </c>
       <c r="D39" t="s">
         <v>24</v>
@@ -2214,27 +2346,27 @@
         <v>25</v>
       </c>
       <c r="F39">
-        <v>130</v>
+        <v>396</v>
       </c>
       <c r="G39" t="s">
-        <v>109</v>
+        <v>178</v>
       </c>
       <c r="H39" t="s">
         <v>27</v>
       </c>
       <c r="I39" t="s">
-        <v>146</v>
+        <v>179</v>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B40" t="s">
-        <v>147</v>
+        <v>180</v>
       </c>
       <c r="C40" t="s">
-        <v>148</v>
+        <v>181</v>
       </c>
       <c r="D40" t="s">
         <v>24</v>
@@ -2243,85 +2375,85 @@
         <v>25</v>
       </c>
       <c r="F40">
-        <v>130</v>
+        <v>452</v>
       </c>
       <c r="G40" t="s">
-        <v>109</v>
+        <v>182</v>
       </c>
       <c r="H40" t="s">
         <v>27</v>
       </c>
       <c r="I40" t="s">
-        <v>149</v>
+        <v>183</v>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B41" t="s">
-        <v>150</v>
+        <v>184</v>
       </c>
       <c r="C41" t="s">
-        <v>151</v>
+        <v>185</v>
       </c>
       <c r="D41" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E41" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F41">
-        <v>131</v>
+        <v>481</v>
       </c>
       <c r="G41" t="s">
-        <v>152</v>
+        <v>186</v>
       </c>
       <c r="H41" t="s">
         <v>27</v>
       </c>
       <c r="I41" t="s">
-        <v>153</v>
+        <v>187</v>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B42" t="s">
-        <v>154</v>
+        <v>188</v>
       </c>
       <c r="C42" t="s">
-        <v>155</v>
+        <v>189</v>
       </c>
       <c r="D42" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E42" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F42">
-        <v>130</v>
+        <v>456</v>
       </c>
       <c r="G42" t="s">
-        <v>152</v>
+        <v>190</v>
       </c>
       <c r="H42" t="s">
         <v>27</v>
       </c>
       <c r="I42" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B43" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="C43" t="s">
-        <v>158</v>
+        <v>193</v>
       </c>
       <c r="D43" t="s">
         <v>24</v>
@@ -2330,85 +2462,85 @@
         <v>25</v>
       </c>
       <c r="F43">
-        <v>130</v>
+        <v>311</v>
       </c>
       <c r="G43" t="s">
-        <v>152</v>
+        <v>194</v>
       </c>
       <c r="H43" t="s">
         <v>27</v>
       </c>
       <c r="I43" t="s">
-        <v>159</v>
+        <v>195</v>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B44" t="s">
-        <v>160</v>
+        <v>196</v>
       </c>
       <c r="C44" t="s">
-        <v>161</v>
+        <v>197</v>
       </c>
       <c r="D44" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E44" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F44">
-        <v>130</v>
+        <v>485</v>
       </c>
       <c r="G44" t="s">
-        <v>152</v>
+        <v>198</v>
       </c>
       <c r="H44" t="s">
         <v>27</v>
       </c>
       <c r="I44" t="s">
-        <v>162</v>
+        <v>199</v>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B45" t="s">
-        <v>163</v>
+        <v>200</v>
       </c>
       <c r="C45" t="s">
-        <v>164</v>
+        <v>201</v>
       </c>
       <c r="D45" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E45" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F45">
-        <v>130</v>
+        <v>284</v>
       </c>
       <c r="G45" t="s">
-        <v>152</v>
+        <v>202</v>
       </c>
       <c r="H45" t="s">
         <v>27</v>
       </c>
       <c r="I45" t="s">
-        <v>165</v>
+        <v>203</v>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B46" t="s">
-        <v>166</v>
+        <v>204</v>
       </c>
       <c r="C46" t="s">
-        <v>167</v>
+        <v>205</v>
       </c>
       <c r="D46" t="s">
         <v>24</v>
@@ -2417,27 +2549,27 @@
         <v>25</v>
       </c>
       <c r="F46">
-        <v>130</v>
+        <v>433</v>
       </c>
       <c r="G46" t="s">
-        <v>152</v>
+        <v>206</v>
       </c>
       <c r="H46" t="s">
         <v>27</v>
       </c>
       <c r="I46" t="s">
-        <v>168</v>
+        <v>207</v>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B47" t="s">
-        <v>169</v>
+        <v>208</v>
       </c>
       <c r="C47" t="s">
-        <v>170</v>
+        <v>209</v>
       </c>
       <c r="D47" t="s">
         <v>24</v>
@@ -2446,56 +2578,56 @@
         <v>25</v>
       </c>
       <c r="F47">
-        <v>130</v>
+        <v>323</v>
       </c>
       <c r="G47" t="s">
-        <v>152</v>
+        <v>210</v>
       </c>
       <c r="H47" t="s">
         <v>27</v>
       </c>
       <c r="I47" t="s">
-        <v>171</v>
+        <v>211</v>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B48" t="s">
-        <v>172</v>
+        <v>212</v>
       </c>
       <c r="C48" t="s">
-        <v>173</v>
+        <v>213</v>
       </c>
       <c r="D48" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E48" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F48">
-        <v>130</v>
+        <v>445</v>
       </c>
       <c r="G48" t="s">
-        <v>152</v>
+        <v>214</v>
       </c>
       <c r="H48" t="s">
         <v>27</v>
       </c>
       <c r="I48" t="s">
-        <v>174</v>
+        <v>215</v>
       </c>
     </row>
     <row r="49" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B49" t="s">
-        <v>175</v>
+        <v>216</v>
       </c>
       <c r="C49" t="s">
-        <v>176</v>
+        <v>217</v>
       </c>
       <c r="D49" t="s">
         <v>24</v>
@@ -2504,27 +2636,27 @@
         <v>25</v>
       </c>
       <c r="F49">
-        <v>130</v>
+        <v>369</v>
       </c>
       <c r="G49" t="s">
-        <v>152</v>
+        <v>218</v>
       </c>
       <c r="H49" t="s">
         <v>27</v>
       </c>
       <c r="I49" t="s">
-        <v>177</v>
+        <v>219</v>
       </c>
     </row>
     <row r="50" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B50" t="s">
-        <v>178</v>
+        <v>220</v>
       </c>
       <c r="C50" t="s">
-        <v>179</v>
+        <v>221</v>
       </c>
       <c r="D50" t="s">
         <v>24</v>
@@ -2533,45 +2665,45 @@
         <v>25</v>
       </c>
       <c r="F50">
-        <v>130</v>
+        <v>313</v>
       </c>
       <c r="G50" t="s">
-        <v>152</v>
+        <v>222</v>
       </c>
       <c r="H50" t="s">
         <v>27</v>
       </c>
       <c r="I50" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B51" t="s">
-        <v>181</v>
+        <v>224</v>
       </c>
       <c r="C51" t="s">
-        <v>182</v>
+        <v>225</v>
       </c>
       <c r="D51" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E51" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F51">
-        <v>130</v>
+        <v>328</v>
       </c>
       <c r="G51" t="s">
-        <v>152</v>
+        <v>226</v>
       </c>
       <c r="H51" t="s">
         <v>27</v>
       </c>
       <c r="I51" t="s">
-        <v>183</v>
+        <v>227</v>
       </c>
     </row>
   </sheetData>

</xml_diff>